<commit_message>
fix: pruebas v2 con flujo RequestTXN + StatusTXN correcto segun especificacion Taecel
</commit_message>
<xml_diff>
--- a/Tabla_Lista_Para_Subir.xlsx
+++ b/Tabla_Lista_Para_Subir.xlsx
@@ -925,25 +925,25 @@
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>2026-05-27 09:24:49</t>
+          <t>2026-05-27 20:12:07</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>260501706296</t>
+          <t>260501761575</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr"/>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>378809</t>
+        </is>
+      </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
           <t>Exitosa</t>
         </is>
       </c>
-      <c r="I2" s="18" t="inlineStr">
-        <is>
-          <t>Consulta Exitosa</t>
-        </is>
-      </c>
+      <c r="I2" s="18" t="n"/>
       <c r="J2" s="12" t="n"/>
       <c r="K2" s="12" t="n"/>
       <c r="L2" s="12" t="n"/>
@@ -981,25 +981,25 @@
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>2026-05-27 09:24:49</t>
+          <t>2026-05-27 20:12:07</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>260501706297</t>
+          <t>260501761590</t>
         </is>
       </c>
-      <c r="G3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>433097</t>
+        </is>
+      </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
           <t>Exitosa</t>
         </is>
       </c>
-      <c r="I3" s="19" t="inlineStr">
-        <is>
-          <t>Consulta Exitosa</t>
-        </is>
-      </c>
+      <c r="I3" s="19" t="n"/>
       <c r="J3" s="12" t="n"/>
       <c r="K3" s="12" t="n"/>
       <c r="L3" s="12" t="n"/>
@@ -1037,25 +1037,25 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>2026-05-27 09:24:49</t>
+          <t>2026-05-27 20:12:07</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>260501706301</t>
+          <t>260501761616</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr"/>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>191566</t>
+        </is>
+      </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
           <t>Exitosa</t>
         </is>
       </c>
-      <c r="I4" s="18" t="inlineStr">
-        <is>
-          <t>Consulta Exitosa</t>
-        </is>
-      </c>
+      <c r="I4" s="18" t="n"/>
       <c r="J4" s="12" t="n"/>
       <c r="K4" s="12" t="n"/>
       <c r="L4" s="12" t="n"/>
@@ -1093,25 +1093,25 @@
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>2026-05-27 09:24:49</t>
+          <t>2026-05-27 20:12:07</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>260501706302</t>
+          <t>260501761634</t>
         </is>
       </c>
-      <c r="G5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>146942</t>
+        </is>
+      </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
           <t>Exitosa</t>
         </is>
       </c>
-      <c r="I5" s="19" t="inlineStr">
-        <is>
-          <t>Consulta Exitosa</t>
-        </is>
-      </c>
+      <c r="I5" s="19" t="n"/>
       <c r="J5" s="12" t="n"/>
       <c r="K5" s="12" t="n"/>
       <c r="L5" s="12" t="n"/>
@@ -1149,25 +1149,21 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>2026-05-27 09:24:49</t>
+          <t>2026-05-27 20:12:07</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>260501706304</t>
+          <t>260501761646</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr"/>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>Exitosa</t>
+          <t>Fracasada</t>
         </is>
       </c>
-      <c r="I6" s="18" t="inlineStr">
-        <is>
-          <t>Consulta Exitosa</t>
-        </is>
-      </c>
+      <c r="I6" s="18" t="n"/>
       <c r="J6" s="12" t="n"/>
       <c r="K6" s="12" t="n"/>
       <c r="L6" s="12" t="n"/>
@@ -1205,25 +1201,25 @@
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>2026-05-27 09:24:49</t>
+          <t>2026-05-27 20:12:07</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>260501706306</t>
+          <t>260501761677</t>
         </is>
       </c>
-      <c r="G7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>198470</t>
+        </is>
+      </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
           <t>Exitosa</t>
         </is>
       </c>
-      <c r="I7" s="19" t="inlineStr">
-        <is>
-          <t>Consulta Exitosa</t>
-        </is>
-      </c>
+      <c r="I7" s="19" t="n"/>
       <c r="J7" s="12" t="n"/>
       <c r="K7" s="12" t="n"/>
       <c r="L7" s="12" t="n"/>
@@ -1261,25 +1257,21 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>2026-05-27 09:24:49</t>
+          <t>2026-05-27 20:12:07</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>260501706310</t>
+          <t>260501761702</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr"/>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Exitosa</t>
+          <t>Fracasada</t>
         </is>
       </c>
-      <c r="I8" s="18" t="inlineStr">
-        <is>
-          <t>Consulta Exitosa</t>
-        </is>
-      </c>
+      <c r="I8" s="18" t="n"/>
       <c r="J8" s="12" t="n"/>
       <c r="K8" s="12" t="n"/>
       <c r="L8" s="12" t="n"/>
@@ -1317,25 +1309,21 @@
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>2026-05-27 09:24:49</t>
+          <t>2026-05-27 20:12:07</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>260501706316</t>
+          <t>260501761753</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr"/>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>Exitosa</t>
+          <t>En proceso</t>
         </is>
       </c>
-      <c r="I9" s="19" t="inlineStr">
-        <is>
-          <t>Consulta Exitosa</t>
-        </is>
-      </c>
+      <c r="I9" s="19" t="n"/>
       <c r="J9" s="12" t="n"/>
       <c r="K9" s="12" t="n"/>
       <c r="L9" s="12" t="n"/>
@@ -1373,25 +1361,21 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>2026-05-27 09:24:49</t>
+          <t>2026-05-27 20:12:07</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>260501706321</t>
+          <t>260501761787</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr"/>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>Exitosa</t>
+          <t>En proceso</t>
         </is>
       </c>
-      <c r="I10" s="18" t="inlineStr">
-        <is>
-          <t>Consulta Exitosa</t>
-        </is>
-      </c>
+      <c r="I10" s="18" t="n"/>
       <c r="J10" s="12" t="n"/>
       <c r="K10" s="12" t="n"/>
       <c r="L10" s="12" t="n"/>
@@ -1429,21 +1413,17 @@
       </c>
       <c r="E11" s="10" t="inlineStr">
         <is>
-          <t>2026-05-27 09:24:49</t>
+          <t>2026-05-27 20:12:07</t>
         </is>
       </c>
       <c r="F11" s="10" t="inlineStr"/>
       <c r="G11" s="10" t="inlineStr"/>
       <c r="H11" s="10" t="inlineStr">
         <is>
-          <t>Exitosa</t>
+          <t>Fracasada</t>
         </is>
       </c>
-      <c r="I11" s="20" t="inlineStr">
-        <is>
-          <t>Tabla de transacciones llena (Código: 3129)</t>
-        </is>
-      </c>
+      <c r="I11" s="20" t="n"/>
       <c r="J11" s="12" t="n"/>
       <c r="K11" s="12" t="n"/>
       <c r="L11" s="12" t="n"/>
@@ -1575,25 +1555,25 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>2026-05-27 09:24:49</t>
+          <t>2026-05-27 20:12:07</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>260501706343</t>
+          <t>260501761835</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr"/>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>657621</t>
+        </is>
+      </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
           <t>Exitosa</t>
         </is>
       </c>
-      <c r="I14" s="18" t="inlineStr">
-        <is>
-          <t>Consulta Exitosa</t>
-        </is>
-      </c>
+      <c r="I14" s="18" t="n"/>
       <c r="J14" s="12" t="n"/>
       <c r="K14" s="12" t="n"/>
       <c r="L14" s="12" t="n"/>
@@ -1633,25 +1613,25 @@
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>2026-05-27 09:24:49</t>
+          <t>2026-05-27 20:12:07</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>260501706351</t>
+          <t>260501761844</t>
         </is>
       </c>
-      <c r="G15" s="7" t="inlineStr"/>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>781601</t>
+        </is>
+      </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
           <t>Exitosa</t>
         </is>
       </c>
-      <c r="I15" s="19" t="inlineStr">
-        <is>
-          <t>Consulta Exitosa</t>
-        </is>
-      </c>
+      <c r="I15" s="19" t="n"/>
       <c r="J15" s="12" t="n"/>
       <c r="K15" s="12" t="n"/>
       <c r="L15" s="12" t="n"/>
@@ -1691,25 +1671,25 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>2026-05-27 09:24:49</t>
+          <t>2026-05-27 20:12:07</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>260501706366</t>
+          <t>260501761850</t>
         </is>
       </c>
-      <c r="G16" s="4" t="inlineStr"/>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>704333</t>
+        </is>
+      </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
           <t>Exitosa</t>
         </is>
       </c>
-      <c r="I16" s="18" t="inlineStr">
-        <is>
-          <t>Consulta Exitosa</t>
-        </is>
-      </c>
+      <c r="I16" s="18" t="n"/>
       <c r="J16" s="12" t="n"/>
       <c r="K16" s="12" t="n"/>
       <c r="L16" s="12" t="n"/>
@@ -1749,25 +1729,25 @@
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>2026-05-27 09:24:49</t>
+          <t>2026-05-27 20:12:07</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>260501706378</t>
+          <t>260501761852</t>
         </is>
       </c>
-      <c r="G17" s="7" t="inlineStr"/>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>289472</t>
+        </is>
+      </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
           <t>Exitosa</t>
         </is>
       </c>
-      <c r="I17" s="19" t="inlineStr">
-        <is>
-          <t>Consulta Exitosa</t>
-        </is>
-      </c>
+      <c r="I17" s="19" t="n"/>
       <c r="J17" s="12" t="n"/>
       <c r="K17" s="12" t="n"/>
       <c r="L17" s="12" t="n"/>
@@ -1807,25 +1787,25 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>2026-05-27 09:24:49</t>
+          <t>2026-05-27 20:12:07</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>260501706396</t>
+          <t>260501761856</t>
         </is>
       </c>
-      <c r="G18" s="4" t="inlineStr"/>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>127468</t>
+        </is>
+      </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
           <t>Exitosa</t>
         </is>
       </c>
-      <c r="I18" s="18" t="inlineStr">
-        <is>
-          <t>Consulta Exitosa</t>
-        </is>
-      </c>
+      <c r="I18" s="18" t="n"/>
       <c r="J18" s="12" t="n"/>
       <c r="K18" s="12" t="n"/>
       <c r="L18" s="12" t="n"/>
@@ -1865,25 +1845,25 @@
       </c>
       <c r="E19" s="10" t="inlineStr">
         <is>
-          <t>2026-05-27 09:24:49</t>
+          <t>2026-05-27 20:12:07</t>
         </is>
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
-          <t>260501706405</t>
+          <t>260501761864</t>
         </is>
       </c>
-      <c r="G19" s="10" t="inlineStr"/>
+      <c r="G19" s="10" t="inlineStr">
+        <is>
+          <t>902628</t>
+        </is>
+      </c>
       <c r="H19" s="10" t="inlineStr">
         <is>
           <t>Exitosa</t>
         </is>
       </c>
-      <c r="I19" s="20" t="inlineStr">
-        <is>
-          <t>Consulta Exitosa</t>
-        </is>
-      </c>
+      <c r="I19" s="20" t="n"/>
       <c r="J19" s="12" t="n"/>
       <c r="K19" s="12" t="n"/>
       <c r="L19" s="12" t="n"/>

</xml_diff>